<commit_message>
create the receipt test and add details to the documentation
</commit_message>
<xml_diff>
--- a/docs/Lab02/Lab02_BBT_TCs_Form.xlsx
+++ b/docs/Lab02/Lab02_BBT_TCs_Form.xlsx
@@ -3,9 +3,9 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29822"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="124226"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D866A412-1C46-44BE-AE29-B62DDEFE2DD9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E4B67165-D2BA-463E-B5CC-F8092C6D8997}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" firstSheet="1" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" firstSheet="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Statement" sheetId="1" r:id="rId1"/>
@@ -93,7 +93,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="202" uniqueCount="100">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="204" uniqueCount="102">
   <si>
     <t>VVSS, Info Romana, 2025-2026</t>
   </si>
@@ -522,6 +522,12 @@
   </si>
   <si>
     <t>" "</t>
+  </si>
+  <si>
+    <t>Temneanu Maria</t>
+  </si>
+  <si>
+    <t>Tapuc Delia</t>
   </si>
 </sst>
 </file>
@@ -1199,7 +1205,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="122">
+  <cellXfs count="116">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
@@ -1285,257 +1291,241 @@
     <xf numFmtId="0" fontId="8" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="33" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="34" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="35" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="36" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="4" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="4" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="2" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="4" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="4" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="3" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="2" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="33" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="34" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="35" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="36" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -1856,12 +1846,12 @@
   </cols>
   <sheetData>
     <row r="1" spans="2:10" x14ac:dyDescent="0.45">
-      <c r="C1" s="48" t="s">
+      <c r="C1" s="52" t="s">
         <v>0</v>
       </c>
-      <c r="D1" s="49"/>
-      <c r="E1" s="49"/>
-      <c r="F1" s="50"/>
+      <c r="D1" s="53"/>
+      <c r="E1" s="53"/>
+      <c r="F1" s="54"/>
       <c r="H1" s="34" t="s">
         <v>1</v>
       </c>
@@ -1869,11 +1859,11 @@
       <c r="J1" s="34"/>
     </row>
     <row r="2" spans="2:10" x14ac:dyDescent="0.45">
-      <c r="H2" s="61" t="s">
+      <c r="H2" s="89" t="s">
         <v>2</v>
       </c>
-      <c r="I2" s="61"/>
-      <c r="J2" s="61"/>
+      <c r="I2" s="89"/>
+      <c r="J2" s="89"/>
     </row>
     <row r="3" spans="2:10" x14ac:dyDescent="0.45">
       <c r="H3" s="2"/>
@@ -1888,15 +1878,23 @@
       <c r="H4" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="I4" s="2"/>
-      <c r="J4" s="2"/>
+      <c r="I4" s="2" t="s">
+        <v>100</v>
+      </c>
+      <c r="J4" s="2">
+        <v>237</v>
+      </c>
     </row>
     <row r="5" spans="2:10" x14ac:dyDescent="0.45">
       <c r="H5" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="I5" s="2"/>
-      <c r="J5" s="2"/>
+      <c r="I5" s="2" t="s">
+        <v>101</v>
+      </c>
+      <c r="J5" s="2">
+        <v>237</v>
+      </c>
     </row>
     <row r="6" spans="2:10" x14ac:dyDescent="0.45">
       <c r="B6" s="20"/>
@@ -2024,21 +2022,21 @@
     </row>
     <row r="24" spans="1:15" ht="14.45" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A24" s="31"/>
-      <c r="B24" s="60" t="s">
+      <c r="B24" s="88" t="s">
         <v>21</v>
       </c>
-      <c r="C24" s="60"/>
-      <c r="D24" s="60"/>
-      <c r="E24" s="60"/>
-      <c r="F24" s="60"/>
-      <c r="G24" s="60"/>
-      <c r="H24" s="60"/>
-      <c r="I24" s="60"/>
-      <c r="J24" s="60"/>
-      <c r="K24" s="60"/>
-      <c r="L24" s="60"/>
-      <c r="M24" s="60"/>
-      <c r="N24" s="60"/>
+      <c r="C24" s="88"/>
+      <c r="D24" s="88"/>
+      <c r="E24" s="88"/>
+      <c r="F24" s="88"/>
+      <c r="G24" s="88"/>
+      <c r="H24" s="88"/>
+      <c r="I24" s="88"/>
+      <c r="J24" s="88"/>
+      <c r="K24" s="88"/>
+      <c r="L24" s="88"/>
+      <c r="M24" s="88"/>
+      <c r="N24" s="88"/>
     </row>
     <row r="26" spans="1:15" x14ac:dyDescent="0.45">
       <c r="C26" s="33"/>
@@ -2078,41 +2076,41 @@
   </cols>
   <sheetData>
     <row r="1" spans="2:17" x14ac:dyDescent="0.45">
-      <c r="B1" s="48" t="s">
+      <c r="B1" s="52" t="s">
         <v>0</v>
       </c>
-      <c r="C1" s="49"/>
-      <c r="D1" s="49"/>
-      <c r="E1" s="50"/>
+      <c r="C1" s="53"/>
+      <c r="D1" s="53"/>
+      <c r="E1" s="54"/>
     </row>
     <row r="3" spans="2:17" x14ac:dyDescent="0.45">
-      <c r="B3" s="100" t="s">
+      <c r="B3" s="91" t="s">
         <v>96</v>
       </c>
-      <c r="C3" s="54"/>
-      <c r="D3" s="54"/>
-      <c r="E3" s="54"/>
-      <c r="F3" s="54"/>
-      <c r="G3" s="55"/>
+      <c r="C3" s="92"/>
+      <c r="D3" s="92"/>
+      <c r="E3" s="92"/>
+      <c r="F3" s="92"/>
+      <c r="G3" s="93"/>
     </row>
     <row r="5" spans="2:17" x14ac:dyDescent="0.45">
-      <c r="B5" s="56" t="s">
+      <c r="B5" s="94" t="s">
         <v>22</v>
       </c>
-      <c r="C5" s="56"/>
-      <c r="D5" s="56"/>
-      <c r="E5" s="56"/>
-      <c r="G5" s="57" t="s">
+      <c r="C5" s="94"/>
+      <c r="D5" s="94"/>
+      <c r="E5" s="94"/>
+      <c r="G5" s="95" t="s">
         <v>23</v>
       </c>
-      <c r="H5" s="57"/>
-      <c r="I5" s="57"/>
-      <c r="J5" s="57"/>
-      <c r="K5" s="57"/>
-      <c r="L5" s="57"/>
-      <c r="M5" s="57"/>
-      <c r="N5" s="57"/>
-      <c r="O5" s="57"/>
+      <c r="H5" s="95"/>
+      <c r="I5" s="95"/>
+      <c r="J5" s="95"/>
+      <c r="K5" s="95"/>
+      <c r="L5" s="95"/>
+      <c r="M5" s="95"/>
+      <c r="N5" s="95"/>
+      <c r="O5" s="95"/>
     </row>
     <row r="6" spans="2:17" x14ac:dyDescent="0.45">
       <c r="B6" s="12" t="s">
@@ -2127,23 +2125,23 @@
       <c r="E6" s="12" t="s">
         <v>27</v>
       </c>
-      <c r="G6" s="58" t="s">
+      <c r="G6" s="66" t="s">
         <v>28</v>
       </c>
-      <c r="H6" s="44" t="s">
+      <c r="H6" s="59" t="s">
         <v>29</v>
       </c>
-      <c r="I6" s="42" t="s">
+      <c r="I6" s="56" t="s">
         <v>30</v>
       </c>
-      <c r="J6" s="47"/>
-      <c r="K6" s="47"/>
-      <c r="L6" s="47"/>
-      <c r="M6" s="47"/>
-      <c r="N6" s="46" t="s">
+      <c r="J6" s="57"/>
+      <c r="K6" s="57"/>
+      <c r="L6" s="57"/>
+      <c r="M6" s="57"/>
+      <c r="N6" s="55" t="s">
         <v>31</v>
       </c>
-      <c r="O6" s="46"/>
+      <c r="O6" s="55"/>
       <c r="P6" s="3"/>
       <c r="Q6" s="3"/>
     </row>
@@ -2151,15 +2149,15 @@
       <c r="B7" s="4">
         <v>1</v>
       </c>
-      <c r="C7" s="51" t="s">
+      <c r="C7" s="90" t="s">
         <v>68</v>
       </c>
       <c r="D7" s="4" t="s">
         <v>69</v>
       </c>
       <c r="E7" s="4"/>
-      <c r="G7" s="59"/>
-      <c r="H7" s="45"/>
+      <c r="G7" s="84"/>
+      <c r="H7" s="98"/>
       <c r="I7" s="12" t="s">
         <v>75</v>
       </c>
@@ -2175,10 +2173,10 @@
       <c r="M7" s="12" t="s">
         <v>78</v>
       </c>
-      <c r="N7" s="42" t="s">
+      <c r="N7" s="56" t="s">
         <v>33</v>
       </c>
-      <c r="O7" s="43"/>
+      <c r="O7" s="58"/>
       <c r="P7" s="3"/>
       <c r="Q7" s="3"/>
     </row>
@@ -2186,12 +2184,12 @@
       <c r="B8" s="4">
         <v>2</v>
       </c>
-      <c r="C8" s="51"/>
+      <c r="C8" s="90"/>
       <c r="D8" s="4"/>
       <c r="E8" s="4" t="s">
         <v>70</v>
       </c>
-      <c r="G8" s="101">
+      <c r="G8" s="37">
         <v>1</v>
       </c>
       <c r="H8" s="35" t="s">
@@ -2212,10 +2210,10 @@
       <c r="M8" s="35" t="s">
         <v>81</v>
       </c>
-      <c r="N8" s="38" t="s">
+      <c r="N8" s="96" t="s">
         <v>34</v>
       </c>
-      <c r="O8" s="39"/>
+      <c r="O8" s="97"/>
       <c r="P8" s="3"/>
       <c r="Q8" s="3"/>
     </row>
@@ -2251,10 +2249,10 @@
       <c r="M9" s="35" t="s">
         <v>81</v>
       </c>
-      <c r="N9" s="38" t="s">
+      <c r="N9" s="96" t="s">
         <v>82</v>
       </c>
-      <c r="O9" s="39"/>
+      <c r="O9" s="97"/>
       <c r="P9" s="3"/>
       <c r="Q9" s="3"/>
     </row>
@@ -2262,7 +2260,7 @@
       <c r="B10" s="4">
         <v>4</v>
       </c>
-      <c r="C10" s="51"/>
+      <c r="C10" s="90"/>
       <c r="D10" s="4"/>
       <c r="E10" s="4" t="s">
         <v>73</v>
@@ -2270,28 +2268,28 @@
       <c r="G10" s="12">
         <v>3</v>
       </c>
-      <c r="H10" s="120" t="s">
+      <c r="H10" s="3" t="s">
         <v>84</v>
       </c>
-      <c r="I10" s="106">
+      <c r="I10" s="35">
         <v>3</v>
       </c>
-      <c r="J10" s="106" t="s">
+      <c r="J10" s="35" t="s">
         <v>85</v>
       </c>
-      <c r="K10" s="106">
+      <c r="K10" s="35">
         <v>-2</v>
       </c>
-      <c r="L10" s="106" t="s">
+      <c r="L10" s="35" t="s">
         <v>80</v>
       </c>
-      <c r="M10" s="106" t="s">
+      <c r="M10" s="35" t="s">
         <v>81</v>
       </c>
-      <c r="N10" s="103" t="s">
+      <c r="N10" s="96" t="s">
         <v>82</v>
       </c>
-      <c r="O10" s="104"/>
+      <c r="O10" s="97"/>
       <c r="P10" s="3"/>
       <c r="Q10" s="3"/>
     </row>
@@ -2299,34 +2297,34 @@
       <c r="B11" s="4">
         <v>10</v>
       </c>
-      <c r="C11" s="51"/>
+      <c r="C11" s="90"/>
       <c r="D11" s="4"/>
       <c r="E11" s="4"/>
       <c r="G11" s="12">
         <v>4</v>
       </c>
-      <c r="H11" s="106" t="s">
+      <c r="H11" s="35" t="s">
         <v>87</v>
       </c>
-      <c r="I11" s="106">
+      <c r="I11" s="35">
         <v>4</v>
       </c>
-      <c r="J11" s="106" t="s">
+      <c r="J11" s="35" t="s">
         <v>37</v>
       </c>
-      <c r="K11" s="106">
+      <c r="K11" s="35">
         <v>0</v>
       </c>
-      <c r="L11" s="106" t="s">
+      <c r="L11" s="35" t="s">
         <v>80</v>
       </c>
-      <c r="M11" s="106" t="s">
+      <c r="M11" s="35" t="s">
         <v>81</v>
       </c>
-      <c r="N11" s="103" t="s">
+      <c r="N11" s="96" t="s">
         <v>82</v>
       </c>
-      <c r="O11" s="104"/>
+      <c r="O11" s="97"/>
       <c r="P11" s="3"/>
       <c r="Q11" s="3"/>
     </row>
@@ -2334,7 +2332,7 @@
       <c r="B12" s="4">
         <v>11</v>
       </c>
-      <c r="C12" s="51"/>
+      <c r="C12" s="90"/>
       <c r="D12" s="4"/>
       <c r="E12" s="4"/>
       <c r="G12" s="11"/>
@@ -2344,14 +2342,14 @@
       <c r="K12" s="10"/>
       <c r="L12" s="10"/>
       <c r="M12" s="10"/>
-      <c r="N12" s="40"/>
-      <c r="O12" s="41"/>
+      <c r="N12" s="100"/>
+      <c r="O12" s="101"/>
     </row>
     <row r="13" spans="2:17" x14ac:dyDescent="0.45">
       <c r="B13" s="4">
         <v>12</v>
       </c>
-      <c r="C13" s="51"/>
+      <c r="C13" s="90"/>
       <c r="D13" s="4"/>
       <c r="E13" s="4"/>
       <c r="G13" s="11"/>
@@ -2361,14 +2359,14 @@
       <c r="K13" s="10"/>
       <c r="L13" s="10"/>
       <c r="M13" s="10"/>
-      <c r="N13" s="40"/>
-      <c r="O13" s="41"/>
+      <c r="N13" s="100"/>
+      <c r="O13" s="101"/>
     </row>
     <row r="14" spans="2:17" x14ac:dyDescent="0.45">
       <c r="B14" s="4">
         <v>13</v>
       </c>
-      <c r="C14" s="51"/>
+      <c r="C14" s="90"/>
       <c r="D14" s="4"/>
       <c r="E14" s="4"/>
       <c r="G14" s="12"/>
@@ -2378,14 +2376,14 @@
       <c r="K14" s="2"/>
       <c r="L14" s="2"/>
       <c r="M14" s="2"/>
-      <c r="N14" s="40"/>
-      <c r="O14" s="41"/>
+      <c r="N14" s="100"/>
+      <c r="O14" s="101"/>
     </row>
     <row r="15" spans="2:17" x14ac:dyDescent="0.45">
       <c r="B15" s="4">
         <v>14</v>
       </c>
-      <c r="C15" s="51"/>
+      <c r="C15" s="90"/>
       <c r="D15" s="4"/>
       <c r="E15" s="4"/>
     </row>
@@ -2393,11 +2391,16 @@
       <c r="D17" t="s">
         <v>38</v>
       </c>
-      <c r="F17" s="37"/>
-      <c r="G17" s="37"/>
+      <c r="F17" s="99"/>
+      <c r="G17" s="99"/>
     </row>
   </sheetData>
   <mergeCells count="21">
+    <mergeCell ref="F17:G17"/>
+    <mergeCell ref="N11:O11"/>
+    <mergeCell ref="N12:O12"/>
+    <mergeCell ref="N13:O13"/>
+    <mergeCell ref="N14:O14"/>
     <mergeCell ref="B1:E1"/>
     <mergeCell ref="C14:C15"/>
     <mergeCell ref="C7:C8"/>
@@ -2413,11 +2416,6 @@
     <mergeCell ref="N6:O6"/>
     <mergeCell ref="I6:M6"/>
     <mergeCell ref="N7:O7"/>
-    <mergeCell ref="F17:G17"/>
-    <mergeCell ref="N11:O11"/>
-    <mergeCell ref="N12:O12"/>
-    <mergeCell ref="N13:O13"/>
-    <mergeCell ref="N14:O14"/>
     <mergeCell ref="N10:O10"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -2451,43 +2449,43 @@
   </cols>
   <sheetData>
     <row r="1" spans="2:17" x14ac:dyDescent="0.45">
-      <c r="B1" s="48" t="s">
+      <c r="B1" s="52" t="s">
         <v>0</v>
       </c>
-      <c r="C1" s="49"/>
-      <c r="D1" s="49"/>
-      <c r="E1" s="50"/>
+      <c r="C1" s="53"/>
+      <c r="D1" s="53"/>
+      <c r="E1" s="54"/>
     </row>
     <row r="3" spans="2:17" x14ac:dyDescent="0.45">
-      <c r="B3" s="100" t="s">
+      <c r="B3" s="91" t="s">
         <v>83</v>
       </c>
-      <c r="C3" s="54"/>
-      <c r="D3" s="54"/>
-      <c r="E3" s="54"/>
-      <c r="F3" s="54"/>
-      <c r="G3" s="55"/>
+      <c r="C3" s="92"/>
+      <c r="D3" s="92"/>
+      <c r="E3" s="92"/>
+      <c r="F3" s="92"/>
+      <c r="G3" s="93"/>
     </row>
     <row r="5" spans="2:17" x14ac:dyDescent="0.45">
-      <c r="B5" s="68" t="s">
+      <c r="B5" s="110" t="s">
         <v>39</v>
       </c>
-      <c r="C5" s="68"/>
-      <c r="D5" s="68"/>
+      <c r="C5" s="110"/>
+      <c r="D5" s="110"/>
       <c r="E5" s="3"/>
-      <c r="G5" s="57" t="s">
+      <c r="G5" s="95" t="s">
         <v>40</v>
       </c>
-      <c r="H5" s="57"/>
-      <c r="I5" s="57"/>
-      <c r="J5" s="57"/>
-      <c r="K5" s="57"/>
-      <c r="L5" s="57"/>
-      <c r="M5" s="57"/>
-      <c r="N5" s="57"/>
-      <c r="O5" s="57"/>
-      <c r="P5" s="57"/>
-      <c r="Q5" s="57"/>
+      <c r="H5" s="95"/>
+      <c r="I5" s="95"/>
+      <c r="J5" s="95"/>
+      <c r="K5" s="95"/>
+      <c r="L5" s="95"/>
+      <c r="M5" s="95"/>
+      <c r="N5" s="95"/>
+      <c r="O5" s="95"/>
+      <c r="P5" s="95"/>
+      <c r="Q5" s="95"/>
     </row>
     <row r="6" spans="2:17" ht="14.45" customHeight="1" x14ac:dyDescent="0.45">
       <c r="B6" s="4" t="s">
@@ -2501,45 +2499,45 @@
       </c>
       <c r="E6" s="6"/>
       <c r="F6" s="3"/>
-      <c r="G6" s="58" t="s">
+      <c r="G6" s="66" t="s">
         <v>42</v>
       </c>
-      <c r="H6" s="58" t="s">
+      <c r="H6" s="66" t="s">
         <v>43</v>
       </c>
-      <c r="I6" s="58" t="s">
+      <c r="I6" s="66" t="s">
         <v>44</v>
       </c>
-      <c r="J6" s="44" t="s">
+      <c r="J6" s="59" t="s">
         <v>45</v>
       </c>
-      <c r="K6" s="64" t="s">
+      <c r="K6" s="111" t="s">
         <v>30</v>
       </c>
-      <c r="L6" s="65"/>
-      <c r="M6" s="65"/>
-      <c r="N6" s="65"/>
-      <c r="O6" s="65"/>
-      <c r="P6" s="64" t="s">
+      <c r="L6" s="113"/>
+      <c r="M6" s="113"/>
+      <c r="N6" s="113"/>
+      <c r="O6" s="113"/>
+      <c r="P6" s="111" t="s">
         <v>31</v>
       </c>
-      <c r="Q6" s="66"/>
+      <c r="Q6" s="112"/>
     </row>
     <row r="7" spans="2:17" x14ac:dyDescent="0.45">
-      <c r="B7" s="52">
+      <c r="B7" s="106">
         <v>1</v>
       </c>
-      <c r="C7" s="70" t="s">
+      <c r="C7" s="107" t="s">
         <v>88</v>
       </c>
       <c r="D7" s="2" t="s">
         <v>89</v>
       </c>
       <c r="F7" s="3"/>
-      <c r="G7" s="59"/>
-      <c r="H7" s="59"/>
-      <c r="I7" s="59"/>
-      <c r="J7" s="45"/>
+      <c r="G7" s="84"/>
+      <c r="H7" s="84"/>
+      <c r="I7" s="84"/>
+      <c r="J7" s="98"/>
       <c r="K7" s="12" t="s">
         <v>75</v>
       </c>
@@ -2555,14 +2553,14 @@
       <c r="O7" s="12" t="s">
         <v>78</v>
       </c>
-      <c r="P7" s="42" t="s">
+      <c r="P7" s="56" t="s">
         <v>46</v>
       </c>
-      <c r="Q7" s="43"/>
+      <c r="Q7" s="58"/>
     </row>
     <row r="8" spans="2:17" x14ac:dyDescent="0.45">
-      <c r="B8" s="69"/>
-      <c r="C8" s="71"/>
+      <c r="B8" s="102"/>
+      <c r="C8" s="104"/>
       <c r="D8" s="2" t="s">
         <v>90</v>
       </c>
@@ -2570,38 +2568,38 @@
       <c r="G8" s="12" t="s">
         <v>93</v>
       </c>
-      <c r="H8" s="105">
+      <c r="H8" s="4">
         <v>1</v>
       </c>
-      <c r="I8" s="106" t="s">
+      <c r="I8" s="35" t="s">
         <v>36</v>
       </c>
-      <c r="J8" s="106" t="s">
+      <c r="J8" s="35" t="s">
         <v>94</v>
       </c>
-      <c r="K8" s="106">
+      <c r="K8" s="35">
         <v>3</v>
       </c>
-      <c r="L8" s="106" t="s">
+      <c r="L8" s="35" t="s">
         <v>79</v>
       </c>
-      <c r="M8" s="106">
+      <c r="M8" s="35">
         <v>0.01</v>
       </c>
-      <c r="N8" s="106" t="s">
+      <c r="N8" s="35" t="s">
         <v>80</v>
       </c>
-      <c r="O8" s="106" t="s">
+      <c r="O8" s="35" t="s">
         <v>81</v>
       </c>
-      <c r="P8" s="103" t="s">
+      <c r="P8" s="96" t="s">
         <v>34</v>
       </c>
-      <c r="Q8" s="104"/>
+      <c r="Q8" s="97"/>
     </row>
     <row r="9" spans="2:17" x14ac:dyDescent="0.45">
-      <c r="B9" s="69"/>
-      <c r="C9" s="71"/>
+      <c r="B9" s="102"/>
+      <c r="C9" s="104"/>
       <c r="D9" s="2" t="s">
         <v>91</v>
       </c>
@@ -2609,38 +2607,38 @@
       <c r="G9" s="12" t="s">
         <v>95</v>
       </c>
-      <c r="H9" s="105">
+      <c r="H9" s="4">
         <v>2</v>
       </c>
-      <c r="I9" s="106" t="s">
+      <c r="I9" s="35" t="s">
         <v>36</v>
       </c>
-      <c r="J9" s="106" t="s">
+      <c r="J9" s="35" t="s">
         <v>94</v>
       </c>
-      <c r="K9" s="106">
+      <c r="K9" s="35">
         <v>4</v>
       </c>
-      <c r="L9" s="106" t="s">
+      <c r="L9" s="35" t="s">
         <v>79</v>
       </c>
-      <c r="M9" s="106">
+      <c r="M9" s="35">
         <v>0</v>
       </c>
-      <c r="N9" s="106" t="s">
+      <c r="N9" s="35" t="s">
         <v>80</v>
       </c>
-      <c r="O9" s="106" t="s">
+      <c r="O9" s="35" t="s">
         <v>81</v>
       </c>
-      <c r="P9" s="103" t="s">
+      <c r="P9" s="96" t="s">
         <v>82</v>
       </c>
-      <c r="Q9" s="104"/>
+      <c r="Q9" s="97"/>
     </row>
     <row r="10" spans="2:17" x14ac:dyDescent="0.45">
-      <c r="B10" s="69"/>
-      <c r="C10" s="71"/>
+      <c r="B10" s="102"/>
+      <c r="C10" s="104"/>
       <c r="D10" s="2" t="s">
         <v>92</v>
       </c>
@@ -2648,75 +2646,75 @@
       <c r="G10" s="12" t="s">
         <v>55</v>
       </c>
-      <c r="H10" s="105">
+      <c r="H10" s="4">
         <v>3</v>
       </c>
-      <c r="I10" s="106" t="s">
+      <c r="I10" s="35" t="s">
         <v>36</v>
       </c>
-      <c r="J10" s="106" t="s">
+      <c r="J10" s="35" t="s">
         <v>94</v>
       </c>
-      <c r="K10" s="106">
+      <c r="K10" s="35">
         <v>5</v>
       </c>
-      <c r="L10" s="106" t="s">
+      <c r="L10" s="35" t="s">
         <v>79</v>
       </c>
-      <c r="M10" s="106">
+      <c r="M10" s="35">
         <v>-0.01</v>
       </c>
-      <c r="N10" s="106" t="s">
+      <c r="N10" s="35" t="s">
         <v>80</v>
       </c>
-      <c r="O10" s="106" t="s">
+      <c r="O10" s="35" t="s">
         <v>81</v>
       </c>
-      <c r="P10" s="103" t="s">
+      <c r="P10" s="96" t="s">
         <v>82</v>
       </c>
-      <c r="Q10" s="104"/>
+      <c r="Q10" s="97"/>
     </row>
     <row r="11" spans="2:17" x14ac:dyDescent="0.45">
-      <c r="B11" s="69"/>
-      <c r="C11" s="71"/>
+      <c r="B11" s="102"/>
+      <c r="C11" s="104"/>
       <c r="D11" s="2"/>
       <c r="F11" s="3"/>
       <c r="G11" s="12" t="s">
         <v>56</v>
       </c>
-      <c r="H11" s="105">
+      <c r="H11" s="4">
         <v>4</v>
       </c>
-      <c r="I11" s="106" t="s">
+      <c r="I11" s="35" t="s">
         <v>54</v>
       </c>
-      <c r="J11" s="106" t="s">
+      <c r="J11" s="35" t="s">
         <v>94</v>
       </c>
-      <c r="K11" s="106">
+      <c r="K11" s="35">
         <v>6</v>
       </c>
-      <c r="L11" s="106" t="s">
+      <c r="L11" s="35" t="s">
         <v>79</v>
       </c>
-      <c r="M11" s="106">
+      <c r="M11" s="35">
         <v>100</v>
       </c>
-      <c r="N11" s="106" t="s">
+      <c r="N11" s="35" t="s">
         <v>80</v>
       </c>
-      <c r="O11" s="106" t="s">
+      <c r="O11" s="35" t="s">
         <v>81</v>
       </c>
-      <c r="P11" s="103" t="s">
+      <c r="P11" s="96" t="s">
         <v>34</v>
       </c>
-      <c r="Q11" s="104"/>
+      <c r="Q11" s="97"/>
     </row>
     <row r="12" spans="2:17" x14ac:dyDescent="0.45">
-      <c r="B12" s="53"/>
-      <c r="C12" s="72"/>
+      <c r="B12" s="103"/>
+      <c r="C12" s="105"/>
       <c r="D12" s="2"/>
       <c r="F12" s="3"/>
       <c r="G12" s="12">
@@ -2730,60 +2728,67 @@
       <c r="M12" s="8"/>
       <c r="N12" s="8"/>
       <c r="O12" s="8"/>
-      <c r="P12" s="62"/>
-      <c r="Q12" s="63"/>
+      <c r="P12" s="114"/>
+      <c r="Q12" s="115"/>
     </row>
     <row r="13" spans="2:17" x14ac:dyDescent="0.45">
-      <c r="B13" s="69"/>
-      <c r="C13" s="71"/>
+      <c r="B13" s="102"/>
+      <c r="C13" s="104"/>
       <c r="D13" s="2" t="s">
         <v>35</v>
       </c>
     </row>
     <row r="14" spans="2:17" x14ac:dyDescent="0.45">
-      <c r="B14" s="69"/>
-      <c r="C14" s="71"/>
+      <c r="B14" s="102"/>
+      <c r="C14" s="104"/>
       <c r="D14" s="2" t="s">
         <v>35</v>
       </c>
     </row>
     <row r="15" spans="2:17" x14ac:dyDescent="0.45">
-      <c r="B15" s="69"/>
-      <c r="C15" s="71"/>
+      <c r="B15" s="102"/>
+      <c r="C15" s="104"/>
       <c r="D15" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="G15" s="37"/>
-      <c r="H15" s="37"/>
-      <c r="I15" s="67"/>
-      <c r="J15" s="67"/>
-      <c r="K15" s="67"/>
-      <c r="L15" s="67"/>
-      <c r="M15" s="67"/>
+      <c r="G15" s="99"/>
+      <c r="H15" s="99"/>
+      <c r="I15" s="109"/>
+      <c r="J15" s="109"/>
+      <c r="K15" s="109"/>
+      <c r="L15" s="109"/>
+      <c r="M15" s="109"/>
       <c r="N15" s="26"/>
     </row>
     <row r="16" spans="2:17" x14ac:dyDescent="0.45">
-      <c r="B16" s="69"/>
-      <c r="C16" s="71"/>
+      <c r="B16" s="102"/>
+      <c r="C16" s="104"/>
       <c r="D16" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="I16" s="73"/>
-      <c r="J16" s="73"/>
-      <c r="K16" s="73"/>
-      <c r="L16" s="73"/>
-      <c r="M16" s="73"/>
+      <c r="I16" s="108"/>
+      <c r="J16" s="108"/>
+      <c r="K16" s="108"/>
+      <c r="L16" s="108"/>
+      <c r="M16" s="108"/>
       <c r="N16" s="27"/>
     </row>
     <row r="17" spans="2:4" x14ac:dyDescent="0.45">
-      <c r="B17" s="53"/>
-      <c r="C17" s="72"/>
+      <c r="B17" s="103"/>
+      <c r="C17" s="105"/>
       <c r="D17" s="2" t="s">
         <v>35</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="23">
+    <mergeCell ref="P11:Q11"/>
+    <mergeCell ref="P12:Q12"/>
+    <mergeCell ref="H6:H7"/>
+    <mergeCell ref="P8:Q8"/>
+    <mergeCell ref="P9:Q9"/>
+    <mergeCell ref="K6:O6"/>
+    <mergeCell ref="P10:Q10"/>
     <mergeCell ref="B1:E1"/>
     <mergeCell ref="G6:G7"/>
     <mergeCell ref="I6:I7"/>
@@ -2800,13 +2805,6 @@
     <mergeCell ref="I15:M15"/>
     <mergeCell ref="B5:D5"/>
     <mergeCell ref="P6:Q6"/>
-    <mergeCell ref="H6:H7"/>
-    <mergeCell ref="P8:Q8"/>
-    <mergeCell ref="P9:Q9"/>
-    <mergeCell ref="K6:O6"/>
-    <mergeCell ref="P10:Q10"/>
-    <mergeCell ref="P11:Q11"/>
-    <mergeCell ref="P12:Q12"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
@@ -2832,66 +2830,66 @@
   </cols>
   <sheetData>
     <row r="1" spans="2:16" x14ac:dyDescent="0.45">
-      <c r="B1" s="48" t="s">
+      <c r="B1" s="52" t="s">
         <v>0</v>
       </c>
-      <c r="C1" s="49"/>
-      <c r="D1" s="49"/>
-      <c r="E1" s="50"/>
+      <c r="C1" s="53"/>
+      <c r="D1" s="53"/>
+      <c r="E1" s="54"/>
     </row>
     <row r="3" spans="2:16" x14ac:dyDescent="0.45">
-      <c r="B3" s="99" t="s">
+      <c r="B3" s="63" t="s">
         <v>47</v>
       </c>
-      <c r="C3" s="99"/>
-      <c r="D3" s="99"/>
-      <c r="E3" s="99"/>
-      <c r="F3" s="99"/>
-      <c r="G3" s="99"/>
-      <c r="H3" s="99"/>
-      <c r="I3" s="99"/>
-      <c r="J3" s="99"/>
-      <c r="K3" s="99"/>
-      <c r="L3" s="99"/>
-      <c r="M3" s="99"/>
-      <c r="N3" s="99"/>
+      <c r="C3" s="63"/>
+      <c r="D3" s="63"/>
+      <c r="E3" s="63"/>
+      <c r="F3" s="63"/>
+      <c r="G3" s="63"/>
+      <c r="H3" s="63"/>
+      <c r="I3" s="63"/>
+      <c r="J3" s="63"/>
+      <c r="K3" s="63"/>
+      <c r="L3" s="63"/>
+      <c r="M3" s="63"/>
+      <c r="N3" s="63"/>
     </row>
     <row r="4" spans="2:16" x14ac:dyDescent="0.45">
-      <c r="B4" s="58" t="s">
+      <c r="B4" s="66" t="s">
         <v>48</v>
       </c>
-      <c r="C4" s="97" t="s">
+      <c r="C4" s="61" t="s">
         <v>49</v>
       </c>
-      <c r="D4" s="85" t="s">
+      <c r="D4" s="45" t="s">
         <v>50</v>
       </c>
-      <c r="E4" s="44" t="s">
+      <c r="E4" s="59" t="s">
         <v>51</v>
       </c>
-      <c r="F4" s="42" t="s">
+      <c r="F4" s="56" t="s">
         <v>30</v>
       </c>
-      <c r="G4" s="47"/>
-      <c r="H4" s="47"/>
-      <c r="I4" s="47"/>
-      <c r="J4" s="47"/>
-      <c r="K4" s="47"/>
-      <c r="L4" s="43"/>
-      <c r="M4" s="46" t="s">
+      <c r="G4" s="57"/>
+      <c r="H4" s="57"/>
+      <c r="I4" s="57"/>
+      <c r="J4" s="57"/>
+      <c r="K4" s="57"/>
+      <c r="L4" s="58"/>
+      <c r="M4" s="55" t="s">
         <v>31</v>
       </c>
-      <c r="N4" s="46"/>
+      <c r="N4" s="55"/>
     </row>
     <row r="5" spans="2:16" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="B5" s="84"/>
-      <c r="C5" s="98"/>
-      <c r="D5" s="86"/>
-      <c r="E5" s="96"/>
+      <c r="B5" s="67"/>
+      <c r="C5" s="62"/>
+      <c r="D5" s="68"/>
+      <c r="E5" s="60"/>
       <c r="F5" s="14" t="s">
         <v>75</v>
       </c>
-      <c r="G5" s="107" t="s">
+      <c r="G5" s="38" t="s">
         <v>76</v>
       </c>
       <c r="H5" s="14" t="s">
@@ -2900,11 +2898,11 @@
       <c r="I5" s="14" t="s">
         <v>32</v>
       </c>
-      <c r="J5" s="110" t="s">
+      <c r="J5" s="43" t="s">
         <v>78</v>
       </c>
-      <c r="K5" s="111"/>
-      <c r="L5" s="85"/>
+      <c r="K5" s="44"/>
+      <c r="L5" s="45"/>
       <c r="M5" s="14" t="s">
         <v>33</v>
       </c>
@@ -2916,7 +2914,7 @@
       <c r="B6" s="13">
         <v>1</v>
       </c>
-      <c r="C6" s="83" t="s">
+      <c r="C6" s="65" t="s">
         <v>53</v>
       </c>
       <c r="D6" s="17" t="s">
@@ -2925,111 +2923,108 @@
       <c r="E6" s="36" t="s">
         <v>36</v>
       </c>
-      <c r="F6" s="118">
+      <c r="F6" s="40">
         <v>1</v>
       </c>
-      <c r="G6" s="118" t="s">
+      <c r="G6" s="40" t="s">
         <v>79</v>
       </c>
-      <c r="H6" s="118">
+      <c r="H6" s="40">
         <v>5</v>
       </c>
-      <c r="I6" s="118" t="s">
+      <c r="I6" s="40" t="s">
         <v>80</v>
       </c>
-      <c r="J6" s="112" t="s">
+      <c r="J6" s="46" t="s">
         <v>81</v>
       </c>
-      <c r="K6" s="113"/>
-      <c r="L6" s="114"/>
+      <c r="K6" s="47"/>
+      <c r="L6" s="48"/>
       <c r="M6" s="36" t="s">
         <v>34</v>
       </c>
       <c r="N6" s="36" t="s">
         <v>34</v>
       </c>
-      <c r="O6" s="102"/>
     </row>
     <row r="7" spans="2:16" x14ac:dyDescent="0.45">
       <c r="B7" s="7">
         <f>B6+1</f>
         <v>2</v>
       </c>
-      <c r="C7" s="83"/>
+      <c r="C7" s="65"/>
       <c r="D7" s="18" t="s">
         <v>97</v>
       </c>
       <c r="E7" s="12" t="s">
         <v>36</v>
       </c>
-      <c r="F7" s="119">
+      <c r="F7" s="41">
         <v>2</v>
       </c>
-      <c r="G7" s="119" t="s">
+      <c r="G7" s="41" t="s">
         <v>37</v>
       </c>
-      <c r="H7" s="119">
+      <c r="H7" s="41">
         <v>10</v>
       </c>
-      <c r="I7" s="121" t="s">
+      <c r="I7" s="42" t="s">
         <v>80</v>
       </c>
-      <c r="J7" s="112" t="s">
+      <c r="J7" s="46" t="s">
         <v>81</v>
       </c>
-      <c r="K7" s="113"/>
-      <c r="L7" s="114"/>
+      <c r="K7" s="47"/>
+      <c r="L7" s="48"/>
       <c r="M7" s="12" t="s">
         <v>82</v>
       </c>
       <c r="N7" s="12" t="s">
         <v>82</v>
       </c>
-      <c r="O7" s="102"/>
     </row>
     <row r="8" spans="2:16" x14ac:dyDescent="0.45">
       <c r="B8" s="7">
         <f t="shared" ref="B8:B11" si="0">B7+1</f>
         <v>3</v>
       </c>
-      <c r="C8" s="83"/>
+      <c r="C8" s="65"/>
       <c r="D8" s="18" t="s">
         <v>98</v>
       </c>
       <c r="E8" s="12" t="s">
         <v>36</v>
       </c>
-      <c r="F8" s="119">
+      <c r="F8" s="41">
         <v>2</v>
       </c>
-      <c r="G8" s="119" t="s">
+      <c r="G8" s="41" t="s">
         <v>99</v>
       </c>
-      <c r="H8" s="119">
+      <c r="H8" s="41">
         <v>10</v>
       </c>
-      <c r="I8" s="121" t="s">
+      <c r="I8" s="42" t="s">
         <v>80</v>
       </c>
-      <c r="J8" s="112" t="s">
+      <c r="J8" s="46" t="s">
         <v>81</v>
       </c>
-      <c r="K8" s="113"/>
-      <c r="L8" s="114"/>
+      <c r="K8" s="47"/>
+      <c r="L8" s="48"/>
       <c r="M8" s="12" t="s">
         <v>82</v>
       </c>
       <c r="N8" s="12" t="s">
         <v>82</v>
       </c>
-      <c r="O8" s="102"/>
     </row>
     <row r="9" spans="2:16" x14ac:dyDescent="0.45">
       <c r="B9" s="7">
         <f t="shared" si="0"/>
         <v>4</v>
       </c>
-      <c r="C9" s="83"/>
+      <c r="C9" s="65"/>
       <c r="D9" s="18" t="s">
         <v>36</v>
       </c>
@@ -3039,101 +3034,98 @@
       <c r="F9" s="12">
         <v>3</v>
       </c>
-      <c r="G9" s="119" t="s">
+      <c r="G9" s="41" t="s">
         <v>79</v>
       </c>
       <c r="H9" s="12">
         <v>0.01</v>
       </c>
-      <c r="I9" s="121" t="s">
+      <c r="I9" s="42" t="s">
         <v>80</v>
       </c>
-      <c r="J9" s="112" t="s">
+      <c r="J9" s="46" t="s">
         <v>81</v>
       </c>
-      <c r="K9" s="113"/>
-      <c r="L9" s="114"/>
+      <c r="K9" s="47"/>
+      <c r="L9" s="48"/>
       <c r="M9" s="12" t="s">
         <v>34</v>
       </c>
       <c r="N9" s="12" t="s">
         <v>34</v>
       </c>
-      <c r="O9" s="102"/>
     </row>
     <row r="10" spans="2:16" x14ac:dyDescent="0.45">
       <c r="B10" s="7">
         <f t="shared" si="0"/>
         <v>5</v>
       </c>
-      <c r="C10" s="83"/>
+      <c r="C10" s="65"/>
       <c r="D10" s="18" t="s">
         <v>36</v>
       </c>
       <c r="E10" s="12" t="s">
         <v>95</v>
       </c>
-      <c r="F10" s="119">
+      <c r="F10" s="41">
         <v>4</v>
       </c>
-      <c r="G10" s="119" t="s">
+      <c r="G10" s="41" t="s">
         <v>79</v>
       </c>
-      <c r="H10" s="119">
+      <c r="H10" s="41">
         <v>0</v>
       </c>
-      <c r="I10" s="121" t="s">
+      <c r="I10" s="42" t="s">
         <v>80</v>
       </c>
-      <c r="J10" s="112" t="s">
+      <c r="J10" s="46" t="s">
         <v>81</v>
       </c>
-      <c r="K10" s="113"/>
-      <c r="L10" s="114"/>
+      <c r="K10" s="47"/>
+      <c r="L10" s="48"/>
       <c r="M10" s="12" t="s">
         <v>82</v>
       </c>
       <c r="N10" s="12" t="s">
         <v>82</v>
       </c>
-      <c r="O10" s="102"/>
     </row>
     <row r="11" spans="2:16" x14ac:dyDescent="0.45">
       <c r="B11" s="7">
         <f t="shared" si="0"/>
         <v>6</v>
       </c>
-      <c r="C11" s="83"/>
+      <c r="C11" s="65"/>
       <c r="D11" s="18" t="s">
         <v>36</v>
       </c>
       <c r="E11" s="12" t="s">
         <v>55</v>
       </c>
-      <c r="F11" s="119">
+      <c r="F11" s="41">
         <v>5</v>
       </c>
-      <c r="G11" s="119" t="s">
+      <c r="G11" s="41" t="s">
         <v>79</v>
       </c>
-      <c r="H11" s="119">
+      <c r="H11" s="41">
         <v>-0.01</v>
       </c>
-      <c r="I11" s="121" t="s">
+      <c r="I11" s="42" t="s">
         <v>80</v>
       </c>
-      <c r="J11" s="115" t="s">
+      <c r="J11" s="49" t="s">
         <v>81</v>
       </c>
-      <c r="K11" s="116"/>
-      <c r="L11" s="117"/>
+      <c r="K11" s="50"/>
+      <c r="L11" s="51"/>
       <c r="M11" s="12" t="s">
         <v>82</v>
       </c>
       <c r="N11" s="12" t="s">
         <v>82</v>
       </c>
-      <c r="O11" s="102"/>
     </row>
     <row r="12" spans="2:16" x14ac:dyDescent="0.45">
       <c r="B12" s="15"/>
@@ -3141,7 +3133,7 @@
       <c r="D12" s="16"/>
       <c r="E12" s="15"/>
       <c r="F12" s="15"/>
-      <c r="G12" s="108"/>
+      <c r="G12" s="39"/>
       <c r="H12" s="15"/>
       <c r="I12" s="15"/>
       <c r="J12" s="15"/>
@@ -3162,76 +3154,76 @@
       <c r="H13" s="5"/>
       <c r="I13" s="5"/>
       <c r="J13" s="5"/>
-      <c r="K13" s="82"/>
-      <c r="L13" s="82"/>
+      <c r="K13" s="64"/>
+      <c r="L13" s="64"/>
       <c r="M13" s="5"/>
     </row>
     <row r="14" spans="2:16" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
       <c r="M14" s="5"/>
     </row>
     <row r="15" spans="2:16" ht="14.65" thickTop="1" x14ac:dyDescent="0.45">
-      <c r="C15" s="76" t="s">
+      <c r="C15" s="75" t="s">
         <v>58</v>
       </c>
-      <c r="D15" s="78"/>
-      <c r="E15" s="78"/>
-      <c r="F15" s="79"/>
+      <c r="D15" s="76"/>
+      <c r="E15" s="76"/>
+      <c r="F15" s="77"/>
       <c r="G15" s="22" t="s">
         <v>59</v>
       </c>
-      <c r="H15" s="76" t="s">
+      <c r="H15" s="75" t="s">
         <v>60</v>
       </c>
-      <c r="I15" s="77"/>
-      <c r="J15" s="78"/>
-      <c r="K15" s="78"/>
-      <c r="L15" s="79"/>
-      <c r="M15" s="76" t="s">
+      <c r="I15" s="78"/>
+      <c r="J15" s="76"/>
+      <c r="K15" s="76"/>
+      <c r="L15" s="77"/>
+      <c r="M15" s="75" t="s">
         <v>61</v>
       </c>
-      <c r="N15" s="77"/>
-      <c r="O15" s="78"/>
-      <c r="P15" s="79"/>
+      <c r="N15" s="78"/>
+      <c r="O15" s="76"/>
+      <c r="P15" s="77"/>
     </row>
     <row r="16" spans="2:16" ht="14.45" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B16" s="89" t="s">
+      <c r="B16" s="71" t="s">
         <v>49</v>
       </c>
-      <c r="C16" s="90" t="s">
+      <c r="C16" s="72" t="s">
         <v>62</v>
       </c>
-      <c r="D16" s="75" t="s">
+      <c r="D16" s="73" t="s">
         <v>63</v>
       </c>
-      <c r="E16" s="75" t="s">
+      <c r="E16" s="73" t="s">
         <v>64</v>
       </c>
       <c r="F16" s="74" t="s">
         <v>65</v>
       </c>
-      <c r="G16" s="95" t="s">
+      <c r="G16" s="83" t="s">
         <v>66</v>
       </c>
-      <c r="H16" s="91" t="s">
+      <c r="H16" s="79" t="s">
         <v>67</v>
       </c>
-      <c r="I16" s="92"/>
-      <c r="J16" s="75" t="s">
+      <c r="I16" s="80"/>
+      <c r="J16" s="73" t="s">
         <v>62</v>
       </c>
-      <c r="K16" s="58" t="s">
+      <c r="K16" s="66" t="s">
         <v>63</v>
       </c>
-      <c r="L16" s="97" t="s">
+      <c r="L16" s="61" t="s">
         <v>64</v>
       </c>
-      <c r="M16" s="80" t="s">
+      <c r="M16" s="86" t="s">
         <v>67</v>
       </c>
-      <c r="N16" s="75" t="s">
+      <c r="N16" s="73" t="s">
         <v>62</v>
       </c>
-      <c r="O16" s="75" t="s">
+      <c r="O16" s="73" t="s">
         <v>63</v>
       </c>
       <c r="P16" s="74" t="s">
@@ -3239,20 +3231,20 @@
       </c>
     </row>
     <row r="17" spans="2:16" x14ac:dyDescent="0.45">
-      <c r="B17" s="89"/>
-      <c r="C17" s="90"/>
-      <c r="D17" s="75"/>
-      <c r="E17" s="75"/>
+      <c r="B17" s="71"/>
+      <c r="C17" s="72"/>
+      <c r="D17" s="73"/>
+      <c r="E17" s="73"/>
       <c r="F17" s="74"/>
-      <c r="G17" s="95"/>
-      <c r="H17" s="93"/>
-      <c r="I17" s="94"/>
-      <c r="J17" s="75"/>
-      <c r="K17" s="59"/>
-      <c r="L17" s="109"/>
-      <c r="M17" s="81"/>
-      <c r="N17" s="75"/>
-      <c r="O17" s="75"/>
+      <c r="G17" s="83"/>
+      <c r="H17" s="81"/>
+      <c r="I17" s="82"/>
+      <c r="J17" s="73"/>
+      <c r="K17" s="84"/>
+      <c r="L17" s="85"/>
+      <c r="M17" s="87"/>
+      <c r="N17" s="73"/>
+      <c r="O17" s="73"/>
       <c r="P17" s="74"/>
     </row>
     <row r="18" spans="2:16" x14ac:dyDescent="0.45">
@@ -3274,10 +3266,10 @@
       <c r="G18" s="29">
         <v>1</v>
       </c>
-      <c r="H18" s="87">
+      <c r="H18" s="69">
         <v>3</v>
       </c>
-      <c r="I18" s="88"/>
+      <c r="I18" s="70"/>
       <c r="J18" s="2">
         <v>3</v>
       </c>
@@ -3305,19 +3297,12 @@
     </row>
   </sheetData>
   <mergeCells count="35">
-    <mergeCell ref="J5:L5"/>
-    <mergeCell ref="J6:L6"/>
-    <mergeCell ref="J7:L7"/>
-    <mergeCell ref="J8:L8"/>
-    <mergeCell ref="J9:L9"/>
-    <mergeCell ref="J10:L10"/>
-    <mergeCell ref="J11:L11"/>
-    <mergeCell ref="B1:E1"/>
-    <mergeCell ref="M4:N4"/>
-    <mergeCell ref="F4:L4"/>
-    <mergeCell ref="E4:E5"/>
-    <mergeCell ref="C4:C5"/>
-    <mergeCell ref="B3:N3"/>
+    <mergeCell ref="L16:L17"/>
+    <mergeCell ref="O16:O17"/>
+    <mergeCell ref="P16:P17"/>
+    <mergeCell ref="M15:P15"/>
+    <mergeCell ref="M16:M17"/>
+    <mergeCell ref="N16:N17"/>
     <mergeCell ref="K13:L13"/>
     <mergeCell ref="C6:C11"/>
     <mergeCell ref="B4:B5"/>
@@ -3334,12 +3319,19 @@
     <mergeCell ref="H16:I17"/>
     <mergeCell ref="G16:G17"/>
     <mergeCell ref="K16:K17"/>
-    <mergeCell ref="L16:L17"/>
-    <mergeCell ref="O16:O17"/>
-    <mergeCell ref="P16:P17"/>
-    <mergeCell ref="M15:P15"/>
-    <mergeCell ref="M16:M17"/>
-    <mergeCell ref="N16:N17"/>
+    <mergeCell ref="J10:L10"/>
+    <mergeCell ref="J11:L11"/>
+    <mergeCell ref="B1:E1"/>
+    <mergeCell ref="M4:N4"/>
+    <mergeCell ref="F4:L4"/>
+    <mergeCell ref="E4:E5"/>
+    <mergeCell ref="C4:C5"/>
+    <mergeCell ref="B3:N3"/>
+    <mergeCell ref="J5:L5"/>
+    <mergeCell ref="J6:L6"/>
+    <mergeCell ref="J7:L7"/>
+    <mergeCell ref="J8:L8"/>
+    <mergeCell ref="J9:L9"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
@@ -3348,18 +3340,18 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
   <Display>DocumentLibraryForm</Display>
   <Edit>DocumentLibraryForm</Edit>
   <New>DocumentLibraryForm</New>
 </FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
@@ -3501,18 +3493,18 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{83B9CA12-8961-4BEB-8D70-94D8CF82FF06}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{47FE877D-432C-44A9-9889-489A1D266CB2}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{47FE877D-432C-44A9-9889-489A1D266CB2}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{83B9CA12-8961-4BEB-8D70-94D8CF82FF06}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>

</xml_diff>